<commit_message>
Complete institutional finance model release
</commit_message>
<xml_diff>
--- a/05_Private_Credit/_template_CREDIT.xlsx
+++ b/05_Private_Credit/_template_CREDIT.xlsx
@@ -8,18 +8,25 @@
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Operating Case" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Debt Schedule" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Covenants" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Yield &amp; Spread" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Recovery" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Sensitivity" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Checks" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Sources" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="RefreshLog" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Institutional Surface" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Challenge Log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Lineage Map" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Assumptions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Operating Case" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Debt Schedule" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Covenants" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Yield &amp; Spread" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Recovery" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Sensitivity" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Checks" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Sources" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="RefreshLog" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="FS_MODEL_ID">'Institutional Surface'!$C$4</definedName>
+    <definedName name="FS_DOMAIN">'Institutional Surface'!$C$5</definedName>
+    <definedName name="FS_MATURITY">'Institutional Surface'!$C$6</definedName>
+  </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
@@ -34,7 +41,7 @@
     <numFmt numFmtId="168" formatCode="0.00%;[Red](0.00%);-"/>
     <numFmt numFmtId="169" formatCode="0 &quot;bps&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -87,8 +94,20 @@
       <color rgb="00008000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="15"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -105,8 +124,18 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0017365D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -124,11 +153,16 @@
         <color rgb="00111827"/>
       </top>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00B7B7B7"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -160,6 +194,15 @@
     <xf numFmtId="169" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -725,6 +768,490 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B2:D13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="28" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Recovery &amp; Loss Analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Bridge</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Downside</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Stressed EBITDA</t>
+        </is>
+      </c>
+      <c r="C5" s="17">
+        <f>'Operating Case'!H7</f>
+        <v/>
+      </c>
+      <c r="D5" s="17">
+        <f>'Operating Case'!H7*(1+Assumptions!D7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Recovery multiple</t>
+        </is>
+      </c>
+      <c r="C6" s="21">
+        <f>Assumptions!C23</f>
+        <v/>
+      </c>
+      <c r="D6" s="21">
+        <f>Assumptions!D23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Gross enterprise value</t>
+        </is>
+      </c>
+      <c r="C7" s="17">
+        <f>C5*C6</f>
+        <v/>
+      </c>
+      <c r="D7" s="17">
+        <f>D5*D6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>EV haircut</t>
+        </is>
+      </c>
+      <c r="C8" s="17">
+        <f>C7*Assumptions!C24</f>
+        <v/>
+      </c>
+      <c r="D8" s="17">
+        <f>D7*Assumptions!D24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Net distributable value</t>
+        </is>
+      </c>
+      <c r="C9" s="17">
+        <f>C7-C8</f>
+        <v/>
+      </c>
+      <c r="D9" s="17">
+        <f>D7-D8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Debt claim</t>
+        </is>
+      </c>
+      <c r="C10" s="17">
+        <f>'Debt Schedule'!H15</f>
+        <v/>
+      </c>
+      <c r="D10" s="17">
+        <f>'Debt Schedule'!H15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>Recovery value</t>
+        </is>
+      </c>
+      <c r="C11" s="20">
+        <f>MIN(C9,C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="20">
+        <f>MIN(D9,D10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Recovery rate</t>
+        </is>
+      </c>
+      <c r="C12" s="18">
+        <f>IFERROR(C11/C10,0)</f>
+        <v/>
+      </c>
+      <c r="D12" s="18">
+        <f>IFERROR(D11/D10,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>LGD</t>
+        </is>
+      </c>
+      <c r="C13" s="18">
+        <f>1-C12</f>
+        <v/>
+      </c>
+      <c r="D13" s="18">
+        <f>1-D12</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="28" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Recovery Sensitivity</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>EBITDA haircut / multiple</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B5)*C$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="D5" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B5)*D$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="E5" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B5)*E$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="F5" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B5)*F$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="G5" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B5)*G$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="18" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C6" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B6)*C$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="D6" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B6)*D$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="E6" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B6)*E$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="F6" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B6)*F$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="G6" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B6)*G$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C7" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B7)*C$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="D7" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B7)*D$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="E7" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B7)*E$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="F7" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B7)*F$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="G7" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B7)*G$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C8" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B8)*C$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="D8" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B8)*D$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="E8" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B8)*E$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="F8" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B8)*F$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="G8" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B8)*G$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C9" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B9)*C$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="D9" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B9)*D$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="E9" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B9)*E$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="F9" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B9)*F$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+      <c r="G9" s="18">
+        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B9)*G$4)/'Debt Schedule'!$H$15)),1)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:G2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C5:G9">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="00FCE4D6"/>
+        <color rgb="00FFF2CC"/>
+        <color rgb="00E2F0D9"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="28" customHeight="1">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Model Checks</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Debt nonnegative</t>
+        </is>
+      </c>
+      <c r="C5">
+        <f>IF(MIN('Debt Schedule'!D15:H15)&gt;=0,"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Cash above minimum</t>
+        </is>
+      </c>
+      <c r="C6">
+        <f>IF(MIN('Debt Schedule'!D10:H10)&gt;=Assumptions!E19,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Recovery bounded</t>
+        </is>
+      </c>
+      <c r="C7">
+        <f>IF(AND(MIN(Recovery!C12:D12)&gt;=0,MAX(Recovery!C12:D12)&lt;=1),"PASS","FAIL")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>No covenant breach</t>
+        </is>
+      </c>
+      <c r="C8">
+        <f>IF(COUNTIF(Covenants!C14:G14,"BREACH")=0,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Overall</t>
+        </is>
+      </c>
+      <c r="C9">
+        <f>IF(COUNTIF(C5:C8,"FAIL")+COUNTIF(C5:C8,"REVIEW")=0,"PASS","REVIEW")</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:C2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="C5:C9">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>C5="PASS"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>C5="FAIL"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="2">
+      <formula>C5="REVIEW"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="1">
+      <formula>C5="BREACH"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -860,7 +1387,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1131,6 +1658,1341 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="B2:F64"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="27" t="inlineStr">
+        <is>
+          <t>Private Credit — Institutional Decision Surface</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="28" t="inlineStr">
+        <is>
+          <t>Model ID</t>
+        </is>
+      </c>
+      <c r="C4" s="29" t="inlineStr">
+        <is>
+          <t>05</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="28" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="C5" s="29" t="inlineStr">
+        <is>
+          <t>Private Credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="28" t="inlineStr">
+        <is>
+          <t>Declared maturity</t>
+        </is>
+      </c>
+      <c r="C6" s="29" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="28" t="inlineStr">
+        <is>
+          <t>Canonical builder</t>
+        </is>
+      </c>
+      <c r="C7" s="29" t="inlineStr">
+        <is>
+          <t>tools/builders/build_private_credit_template.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="28" t="inlineStr">
+        <is>
+          <t>Decision arena</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="inlineStr">
+        <is>
+          <t>origination, underwriting, portfolio management, workout and credit committee</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="28" t="inlineStr">
+        <is>
+          <t>Committee artifact</t>
+        </is>
+      </c>
+      <c r="C9" s="29" t="inlineStr">
+        <is>
+          <t>credit approval memorandum</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="28" t="inlineStr">
+        <is>
+          <t>Operating cadence</t>
+        </is>
+      </c>
+      <c r="C10" s="29" t="inlineStr">
+        <is>
+          <t>weekly watchlist; monthly portfolio; event-driven amendments</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>Key decision outputs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="31" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C13" s="31" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="D13" s="31" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E13" s="31" t="inlineStr">
+        <is>
+          <t>Evidence / location</t>
+        </is>
+      </c>
+      <c r="F13" s="31" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>cash yield, OID and all-in return</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>fixed-charge and interest coverage</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>liquidity runway and revolver use</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" t="n">
+        <v>4</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>base, downside and break-even outputs</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>liquidity / funding requirement and binding constraint</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>Insider questions</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="31" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C21" s="31" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="D21" s="31" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E21" s="31" t="inlineStr">
+        <is>
+          <t>Evidence / location</t>
+        </is>
+      </c>
+      <c r="F21" s="31" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>What add-backs are capped or time-limited?</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Where can new money prime us?</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>What is the first liquidity date, not the maturity date?</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Which assumption is owner-approved versus modeler judgement?</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="n">
+        <v>5</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>What fails first and who must act?</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="30" t="inlineStr">
+        <is>
+          <t>Scenario families</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="31" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C29" s="31" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="D29" s="31" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E29" s="31" t="inlineStr">
+        <is>
+          <t>Evidence / location</t>
+        </is>
+      </c>
+      <c r="F29" s="31" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="n">
+        <v>1</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>EBITDA miss and add-back rejection</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="n">
+        <v>2</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>liquidity draw and revolver block</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="n">
+        <v>3</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>rate shock</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="n">
+        <v>4</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>data freshness / source failure</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="n">
+        <v>5</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>combined severe-but-plausible downside</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="30" t="inlineStr">
+        <is>
+          <t>Primary diligence documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="31" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C37" s="31" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="D37" s="31" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E37" s="31" t="inlineStr">
+        <is>
+          <t>Evidence / location</t>
+        </is>
+      </c>
+      <c r="F37" s="31" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>credit agreement and schedules</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" t="n">
+        <v>2</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>QoE and borrowing-base reports</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" t="n">
+        <v>3</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>sponsor model and lender case</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" t="n">
+        <v>4</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>approved model card and assumption register</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" t="n">
+        <v>5</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>independent validation and challenge record</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="30" t="inlineStr">
+        <is>
+          <t>Challenge tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="31" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C45" s="31" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="D45" s="31" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E45" s="31" t="inlineStr">
+        <is>
+          <t>Evidence / location</t>
+        </is>
+      </c>
+      <c r="F45" s="31" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>debt cash schedule conserves</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="n">
+        <v>2</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>yield includes OID and fees</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="n">
+        <v>3</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>recovery cannot exceed collateral after costs</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="n">
+        <v>4</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>source-to-model lineage is reproducible</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="n">
+        <v>5</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>units, signs, dates and legal definitions reconcile</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="30" t="inlineStr">
+        <is>
+          <t>Known failure modes</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="31" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="C53" s="31" t="inlineStr">
+        <is>
+          <t>Requirement</t>
+        </is>
+      </c>
+      <c r="D53" s="31" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="E53" s="31" t="inlineStr">
+        <is>
+          <t>Evidence / location</t>
+        </is>
+      </c>
+      <c r="F53" s="31" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="n">
+        <v>1</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>underwriting to sponsor EBITDA</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="n">
+        <v>2</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>ignoring builder baskets and incremental debt</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>assuming unrestricted cash is available</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" t="n">
+        <v>4</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>stale vintage presented as current</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="B58" t="n">
+        <v>5</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>decision output disconnected from a binding constraint</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr"/>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" s="30" t="inlineStr">
+        <is>
+          <t>Regulatory / methodological anchors</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" s="31" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="C61" s="31" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="D61" s="31" t="inlineStr">
+        <is>
+          <t>Source URL</t>
+        </is>
+      </c>
+      <c r="E61" s="31" t="inlineStr">
+        <is>
+          <t>Applicability</t>
+        </is>
+      </c>
+      <c r="F61" s="31" t="inlineStr">
+        <is>
+          <t>Review note</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Federal Reserve SR 26-2 Model Risk Management</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>governance, validation, change control, monitoring</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/supervisionreg/srletters/SR2602.htm</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Map explicitly</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>OCC Rating Credit Risk</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>repayment capacity and risk rating</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://www.occ.treas.gov/publications-and-resources/publications/comptrollers-handbook/files/rating-credit-risk/pub-ch-rating-credit-risk.pdf</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Map explicitly</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>FASB CECL</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>lifetime expected credit loss</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://www.fasb.org/page/PageContent?pageId=/projects/recentlycompleted/credit-losses.html</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Map explicitly</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="15">
+    <mergeCell ref="B44:F44"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B28:F28"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="B60:F60"/>
+    <mergeCell ref="B36:F36"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="B52:F52"/>
+  </mergeCells>
+  <dataValidations count="6">
+    <dataValidation sqref="F14:F18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"OPEN,IN REVIEW,CLOSED,NOT APPLICABLE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F22:F26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"OPEN,IN REVIEW,CLOSED,NOT APPLICABLE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F30:F34" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"OPEN,IN REVIEW,CLOSED,NOT APPLICABLE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F38:F42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"OPEN,IN REVIEW,CLOSED,NOT APPLICABLE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F46:F50" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"OPEN,IN REVIEW,CLOSED,NOT APPLICABLE"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F54:F58" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"OPEN,IN REVIEW,CLOSED,NOT APPLICABLE"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:I9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="27" t="inlineStr">
+        <is>
+          <t>Independent Challenge, Override and Closure Log</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C4" s="31" t="inlineStr">
+        <is>
+          <t>Reviewer</t>
+        </is>
+      </c>
+      <c r="D4" s="31" t="inlineStr">
+        <is>
+          <t>Challenge</t>
+        </is>
+      </c>
+      <c r="E4" s="31" t="inlineStr">
+        <is>
+          <t>Owner response</t>
+        </is>
+      </c>
+      <c r="F4" s="31" t="inlineStr">
+        <is>
+          <t>Evidence</t>
+        </is>
+      </c>
+      <c r="G4" s="31" t="inlineStr">
+        <is>
+          <t>Impact</t>
+        </is>
+      </c>
+      <c r="H4" s="31" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I4" s="31" t="inlineStr">
+        <is>
+          <t>Closure</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>debt cash schedule conserves</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>yield includes OID and fees</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>recovery cannot exceed collateral after costs</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>source-to-model lineage is reproducible</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>units, signs, dates and legal definitions reconcile</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:I2"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="H5:H54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"OPEN,IN REVIEW,REMEDIATED,ACCEPTED RISK,CLOSED"</formula1>
+    </dataValidation>
+    <dataValidation sqref="G5:G54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"LOW,MEDIUM,HIGH,CRITICAL"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:J8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="27" t="inlineStr">
+        <is>
+          <t>Source, Transformation, Ownership and Refresh Map</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="31" t="inlineStr">
+        <is>
+          <t>Source class</t>
+        </is>
+      </c>
+      <c r="C4" s="31" t="inlineStr">
+        <is>
+          <t>Cadence</t>
+        </is>
+      </c>
+      <c r="D4" s="31" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="E4" s="31" t="inlineStr">
+        <is>
+          <t>System / provider</t>
+        </is>
+      </c>
+      <c r="F4" s="31" t="inlineStr">
+        <is>
+          <t>As-of</t>
+        </is>
+      </c>
+      <c r="G4" s="31" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="H4" s="31" t="inlineStr">
+        <is>
+          <t>Transform</t>
+        </is>
+      </c>
+      <c r="I4" s="31" t="inlineStr">
+        <is>
+          <t>Downstream</t>
+        </is>
+      </c>
+      <c r="J4" s="31" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>borrower reporting</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>monthly/quarterly</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>covenant-definition normalization</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>TO MAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>agent notices</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>event-driven</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>principal, interest and amendment log</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>TO MAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>model governance evidence</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>per release</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>version, reviewer, sign-off and change log</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>TO MAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>decision-use snapshot</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>per decision</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>immutable as-of date and source receipt</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>TO MAP</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B2:J2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="J5:J40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"TO MAP,ACTIVE,STALE,EXCEPTION,RETIRED"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="B2:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1646,7 +3508,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2001,7 +3863,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2475,7 +4337,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2824,7 +4686,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3043,488 +4905,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B2:D13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="36" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="2" ht="28" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Recovery &amp; Loss Analysis</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>Bridge</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Base</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>Downside</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Stressed EBITDA</t>
-        </is>
-      </c>
-      <c r="C5" s="17">
-        <f>'Operating Case'!H7</f>
-        <v/>
-      </c>
-      <c r="D5" s="17">
-        <f>'Operating Case'!H7*(1+Assumptions!D7)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Recovery multiple</t>
-        </is>
-      </c>
-      <c r="C6" s="21">
-        <f>Assumptions!C23</f>
-        <v/>
-      </c>
-      <c r="D6" s="21">
-        <f>Assumptions!D23</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Gross enterprise value</t>
-        </is>
-      </c>
-      <c r="C7" s="17">
-        <f>C5*C6</f>
-        <v/>
-      </c>
-      <c r="D7" s="17">
-        <f>D5*D6</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>EV haircut</t>
-        </is>
-      </c>
-      <c r="C8" s="17">
-        <f>C7*Assumptions!C24</f>
-        <v/>
-      </c>
-      <c r="D8" s="17">
-        <f>D7*Assumptions!D24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Net distributable value</t>
-        </is>
-      </c>
-      <c r="C9" s="17">
-        <f>C7-C8</f>
-        <v/>
-      </c>
-      <c r="D9" s="17">
-        <f>D7-D8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Debt claim</t>
-        </is>
-      </c>
-      <c r="C10" s="17">
-        <f>'Debt Schedule'!H15</f>
-        <v/>
-      </c>
-      <c r="D10" s="17">
-        <f>'Debt Schedule'!H15</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="19" t="inlineStr">
-        <is>
-          <t>Recovery value</t>
-        </is>
-      </c>
-      <c r="C11" s="20">
-        <f>MIN(C9,C10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="20">
-        <f>MIN(D9,D10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Recovery rate</t>
-        </is>
-      </c>
-      <c r="C12" s="18">
-        <f>IFERROR(C11/C10,0)</f>
-        <v/>
-      </c>
-      <c r="D12" s="18">
-        <f>IFERROR(D11/D10,0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>LGD</t>
-        </is>
-      </c>
-      <c r="C13" s="18">
-        <f>1-C12</f>
-        <v/>
-      </c>
-      <c r="D13" s="18">
-        <f>1-D12</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B2:D2"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B2:G9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="2" ht="28" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Recovery Sensitivity</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>EBITDA haircut / multiple</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="D4" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="E4" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="F4" s="8" t="n">
-        <v>6</v>
-      </c>
-      <c r="G4" s="8" t="n">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="18" t="n">
-        <v>0</v>
-      </c>
-      <c r="C5" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B5)*C$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="D5" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B5)*D$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="E5" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B5)*E$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="F5" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B5)*F$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="G5" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B5)*G$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="18" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C6" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B6)*C$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="D6" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B6)*D$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="E6" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B6)*E$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="F6" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B6)*F$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="G6" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B6)*G$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="18" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C7" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B7)*C$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="D7" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B7)*D$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="E7" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B7)*E$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="F7" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B7)*F$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="G7" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B7)*G$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" s="18" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C8" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B8)*C$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="D8" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B8)*D$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="E8" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B8)*E$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="F8" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B8)*F$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="G8" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B8)*G$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="18" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="C9" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B9)*C$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="D9" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B9)*D$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="E9" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B9)*E$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="F9" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B9)*F$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-      <c r="G9" s="18">
-        <f>IFERROR(MIN(1,MAX(0,('Operating Case'!$H$7*(1-$B9)*G$4)/'Debt Schedule'!$H$15)),1)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B2:G2"/>
-  </mergeCells>
-  <conditionalFormatting sqref="C5:G9">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="00FCE4D6"/>
-        <color rgb="00FFF2CC"/>
-        <color rgb="00E2F0D9"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="B2:C9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="2" ht="28" customHeight="1">
-      <c r="B2" s="1" t="inlineStr">
-        <is>
-          <t>Model Checks</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Debt nonnegative</t>
-        </is>
-      </c>
-      <c r="C5">
-        <f>IF(MIN('Debt Schedule'!D15:H15)&gt;=0,"PASS","FAIL")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Cash above minimum</t>
-        </is>
-      </c>
-      <c r="C6">
-        <f>IF(MIN('Debt Schedule'!D10:H10)&gt;=Assumptions!E19,"PASS","REVIEW")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Recovery bounded</t>
-        </is>
-      </c>
-      <c r="C7">
-        <f>IF(AND(MIN(Recovery!C12:D12)&gt;=0,MAX(Recovery!C12:D12)&lt;=1),"PASS","FAIL")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>No covenant breach</t>
-        </is>
-      </c>
-      <c r="C8">
-        <f>IF(COUNTIF(Covenants!C14:G14,"BREACH")=0,"PASS","REVIEW")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Overall</t>
-        </is>
-      </c>
-      <c r="C9">
-        <f>IF(COUNTIF(C5:C8,"FAIL")+COUNTIF(C5:C8,"REVIEW")=0,"PASS","REVIEW")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="B2:C2"/>
-  </mergeCells>
-  <conditionalFormatting sqref="C5:C9">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>C5="PASS"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="2" dxfId="1">
-      <formula>C5="FAIL"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="3" dxfId="2">
-      <formula>C5="REVIEW"</formula>
-    </cfRule>
-    <cfRule type="expression" priority="4" dxfId="1">
-      <formula>C5="BREACH"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>